<commit_message>
training of model_comb 3
</commit_message>
<xml_diff>
--- a/model_comb3/EvalOutputs/TestDataset1_predictions_txt.xlsx
+++ b/model_comb3/EvalOutputs/TestDataset1_predictions_txt.xlsx
@@ -478,25 +478,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>111.16</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>111.41</v>
       </c>
       <c r="F2" t="n">
-        <v>224</v>
+        <v>112.89</v>
       </c>
       <c r="G2" t="n">
-        <v>224</v>
+        <v>112.59</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2595</v>
+        <v>0.0002</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -512,25 +512,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>111.11</v>
       </c>
       <c r="F3" t="n">
-        <v>224</v>
+        <v>112.81</v>
       </c>
       <c r="G3" t="n">
-        <v>224</v>
+        <v>111.74</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>0.3935</v>
       </c>
       <c r="I3" t="n">
-        <v>0.161</v>
+        <v>0.0003</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -549,22 +549,22 @@
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>109.52</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>112.48</v>
       </c>
       <c r="F4" t="n">
-        <v>224</v>
+        <v>113.84</v>
       </c>
       <c r="G4" t="n">
-        <v>224</v>
+        <v>113.02</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9764</v>
+        <v>0.0221</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0305</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -580,25 +580,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>110.01</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>111.77</v>
       </c>
       <c r="F5" t="n">
-        <v>224</v>
+        <v>112.51</v>
       </c>
       <c r="G5" t="n">
-        <v>224</v>
+        <v>112.47</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0001</v>
+        <v>0.136</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0772</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -614,25 +614,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>166.5</v>
+        <v>108.78</v>
       </c>
       <c r="E6" t="n">
-        <v>98.20999999999999</v>
+        <v>112.08</v>
       </c>
       <c r="F6" t="n">
-        <v>204.3</v>
+        <v>114.24</v>
       </c>
       <c r="G6" t="n">
-        <v>157.79</v>
+        <v>113.51</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -648,19 +648,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>6.25</v>
+        <v>109.38</v>
       </c>
       <c r="E7" t="n">
-        <v>26.41</v>
+        <v>113.22</v>
       </c>
       <c r="F7" t="n">
-        <v>60.31</v>
+        <v>111.7</v>
       </c>
       <c r="G7" t="n">
-        <v>63.74</v>
+        <v>113.56</v>
       </c>
       <c r="H7" t="n">
         <v>0.0001</v>
@@ -682,25 +682,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>109.59</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>114.18</v>
       </c>
       <c r="F8" t="n">
-        <v>224</v>
+        <v>112.5</v>
       </c>
       <c r="G8" t="n">
-        <v>224</v>
+        <v>114.23</v>
       </c>
       <c r="H8" t="n">
-        <v>0.9999</v>
+        <v>0.999</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0105</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -716,25 +716,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>108.78</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>112.82</v>
       </c>
       <c r="F9" t="n">
-        <v>224</v>
+        <v>113.78</v>
       </c>
       <c r="G9" t="n">
-        <v>224</v>
+        <v>113.12</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.1512</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1451</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -750,25 +750,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>108.82</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>112.9</v>
       </c>
       <c r="F10" t="n">
-        <v>224</v>
+        <v>114.75</v>
       </c>
       <c r="G10" t="n">
-        <v>224</v>
+        <v>113.78</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0005</v>
+        <v>0.0001</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0045</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -784,25 +784,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>109.47</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>112.79</v>
       </c>
       <c r="F11" t="n">
-        <v>224</v>
+        <v>113.96</v>
       </c>
       <c r="G11" t="n">
-        <v>224</v>
+        <v>113.66</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I11" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -818,28 +818,28 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>110.84</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>112.67</v>
       </c>
       <c r="F12" t="n">
-        <v>224</v>
+        <v>112.68</v>
       </c>
       <c r="G12" t="n">
-        <v>224</v>
+        <v>113.28</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>0.0009</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1148</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>0.1915</v>
       </c>
     </row>
     <row r="13">
@@ -852,25 +852,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>110.21</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>112.03</v>
       </c>
       <c r="F13" t="n">
-        <v>224</v>
+        <v>114.24</v>
       </c>
       <c r="G13" t="n">
-        <v>224</v>
+        <v>112.45</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -886,25 +886,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>109.99</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>111.83</v>
       </c>
       <c r="F14" t="n">
-        <v>224</v>
+        <v>113.65</v>
       </c>
       <c r="G14" t="n">
-        <v>224</v>
+        <v>112.26</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>0.3619</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0145</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -920,25 +920,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>108.11</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>112.19</v>
       </c>
       <c r="F15" t="n">
-        <v>224</v>
+        <v>114.27</v>
       </c>
       <c r="G15" t="n">
-        <v>224</v>
+        <v>112.55</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0036</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -954,25 +954,25 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>109.08</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>112.54</v>
       </c>
       <c r="F16" t="n">
-        <v>224</v>
+        <v>113.35</v>
       </c>
       <c r="G16" t="n">
-        <v>224</v>
+        <v>112.64</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0.0052</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -991,25 +991,25 @@
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>109.52</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>112.48</v>
       </c>
       <c r="F17" t="n">
-        <v>224</v>
+        <v>113.84</v>
       </c>
       <c r="G17" t="n">
-        <v>224</v>
+        <v>113.02</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9764</v>
+        <v>0.0221</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1402</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>0.06469999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -1022,28 +1022,28 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>179.86</v>
+        <v>108.52</v>
       </c>
       <c r="E18" t="n">
-        <v>83.77</v>
+        <v>111.48</v>
       </c>
       <c r="F18" t="n">
-        <v>207.82</v>
+        <v>113.14</v>
       </c>
       <c r="G18" t="n">
-        <v>122.29</v>
+        <v>112.73</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8929</v>
+        <v>0.8263</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>0.0384</v>
       </c>
     </row>
     <row r="19">
@@ -1056,28 +1056,28 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>110.01</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>111.77</v>
       </c>
       <c r="F19" t="n">
-        <v>224</v>
+        <v>112.51</v>
       </c>
       <c r="G19" t="n">
-        <v>224</v>
+        <v>112.47</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0001</v>
+        <v>0.136</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0756</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>0.0202</v>
       </c>
     </row>
     <row r="20">
@@ -1090,25 +1090,25 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>110.21</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>111.76</v>
       </c>
       <c r="F20" t="n">
-        <v>224</v>
+        <v>113.07</v>
       </c>
       <c r="G20" t="n">
-        <v>224</v>
+        <v>112.57</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0001</v>
+        <v>0.0215</v>
       </c>
       <c r="I20" t="n">
-        <v>0.044</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1124,25 +1124,25 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>109.51</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>111.55</v>
       </c>
       <c r="F21" t="n">
-        <v>224</v>
+        <v>116.06</v>
       </c>
       <c r="G21" t="n">
-        <v>224</v>
+        <v>113.35</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0.0058</v>
+        <v>0.0025</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1161,25 +1161,25 @@
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>108.03</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>112.9</v>
       </c>
       <c r="F22" t="n">
-        <v>224</v>
+        <v>112.64</v>
       </c>
       <c r="G22" t="n">
-        <v>224</v>
+        <v>113.43</v>
       </c>
       <c r="H22" t="n">
-        <v>0.368</v>
+        <v>0.9999</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1802</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>0.1712</v>
       </c>
     </row>
     <row r="23">
@@ -1195,25 +1195,25 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>108.94</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>111.95</v>
       </c>
       <c r="F23" t="n">
-        <v>224</v>
+        <v>113.85</v>
       </c>
       <c r="G23" t="n">
-        <v>224</v>
+        <v>113.38</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9553</v>
+        <v>0.0905</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1817</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>0.3652</v>
       </c>
     </row>
     <row r="24">
@@ -1226,28 +1226,28 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>109.28</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>111.54</v>
       </c>
       <c r="F24" t="n">
-        <v>224</v>
+        <v>113.81</v>
       </c>
       <c r="G24" t="n">
-        <v>224</v>
+        <v>113.05</v>
       </c>
       <c r="H24" t="n">
-        <v>0.5125</v>
+        <v>0.9992</v>
       </c>
       <c r="I24" t="n">
-        <v>0.1681</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>0.2603</v>
       </c>
     </row>
     <row r="25">
@@ -1263,25 +1263,25 @@
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>108.94</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>111.69</v>
       </c>
       <c r="F25" t="n">
-        <v>224</v>
+        <v>113.21</v>
       </c>
       <c r="G25" t="n">
-        <v>224</v>
+        <v>113.27</v>
       </c>
       <c r="H25" t="n">
-        <v>0.4017</v>
+        <v>0.9436</v>
       </c>
       <c r="I25" t="n">
-        <v>0.1339</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>0.2444</v>
       </c>
     </row>
     <row r="26">
@@ -1294,25 +1294,25 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>110.58</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>111.6</v>
       </c>
       <c r="F26" t="n">
-        <v>224</v>
+        <v>113.1</v>
       </c>
       <c r="G26" t="n">
-        <v>224</v>
+        <v>112.54</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I26" t="n">
-        <v>0.0092</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1328,25 +1328,25 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>110.31</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>112.26</v>
       </c>
       <c r="F27" t="n">
-        <v>224</v>
+        <v>113.95</v>
       </c>
       <c r="G27" t="n">
-        <v>224</v>
+        <v>112.68</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0042</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1362,25 +1362,25 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>110.71</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>112.49</v>
       </c>
       <c r="F28" t="n">
-        <v>224</v>
+        <v>113.14</v>
       </c>
       <c r="G28" t="n">
-        <v>224</v>
+        <v>113.3</v>
       </c>
       <c r="H28" t="n">
-        <v>0.9995000000000001</v>
+        <v>0.9737</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0106</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1396,28 +1396,28 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>110.69</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>112.12</v>
       </c>
       <c r="F29" t="n">
-        <v>224</v>
+        <v>112.36</v>
       </c>
       <c r="G29" t="n">
-        <v>224</v>
+        <v>113.47</v>
       </c>
       <c r="H29" t="n">
-        <v>0.9993</v>
+        <v>0.9992</v>
       </c>
       <c r="I29" t="n">
-        <v>0.0124</v>
+        <v>0.0003</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>0.4557</v>
       </c>
     </row>
     <row r="30">
@@ -1430,25 +1430,25 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>110.9</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>111.13</v>
       </c>
       <c r="F30" t="n">
-        <v>224</v>
+        <v>111.84</v>
       </c>
       <c r="G30" t="n">
-        <v>224</v>
+        <v>112.45</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>0.9999</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0352</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1464,28 +1464,28 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>110.1</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>111.29</v>
       </c>
       <c r="F31" t="n">
-        <v>224</v>
+        <v>113.4</v>
       </c>
       <c r="G31" t="n">
-        <v>224</v>
+        <v>112.11</v>
       </c>
       <c r="H31" t="n">
-        <v>0.9973</v>
+        <v>0.9918</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0459</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>0.2218</v>
       </c>
     </row>
     <row r="32">
@@ -1498,28 +1498,28 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>110.99</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>111.75</v>
       </c>
       <c r="F32" t="n">
-        <v>224</v>
+        <v>113.04</v>
       </c>
       <c r="G32" t="n">
-        <v>224</v>
+        <v>113.83</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1301</v>
+        <v>0.0001</v>
       </c>
       <c r="J32" t="n">
-        <v>0.0022</v>
+        <v>0.1507</v>
       </c>
     </row>
     <row r="33">
@@ -1532,28 +1532,28 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>110.98</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>113.34</v>
       </c>
       <c r="F33" t="n">
-        <v>224</v>
+        <v>111.28</v>
       </c>
       <c r="G33" t="n">
-        <v>224</v>
+        <v>115.11</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>0.0682</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0327</v>
+        <v>0.2761</v>
       </c>
     </row>
     <row r="34">
@@ -1566,28 +1566,28 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>108.14</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>112.3</v>
       </c>
       <c r="F34" t="n">
-        <v>224</v>
+        <v>110.13</v>
       </c>
       <c r="G34" t="n">
-        <v>224</v>
+        <v>115.35</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1276</v>
+        <v>0.001</v>
       </c>
       <c r="J34" t="n">
-        <v>0.0934</v>
+        <v>0.7541</v>
       </c>
     </row>
     <row r="35">
@@ -1600,28 +1600,28 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>109.18</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>112.63</v>
       </c>
       <c r="F35" t="n">
-        <v>224</v>
+        <v>111.43</v>
       </c>
       <c r="G35" t="n">
-        <v>224</v>
+        <v>114.84</v>
       </c>
       <c r="H35" t="n">
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0.2522</v>
+        <v>0.0004</v>
       </c>
       <c r="J35" t="n">
-        <v>0.044</v>
+        <v>0.6079</v>
       </c>
     </row>
     <row r="36">
@@ -1634,28 +1634,28 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>107.49</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>112.91</v>
       </c>
       <c r="F36" t="n">
-        <v>224</v>
+        <v>110.32</v>
       </c>
       <c r="G36" t="n">
-        <v>224</v>
+        <v>113.15</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>0.0711</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>0.5696</v>
       </c>
     </row>
     <row r="37">
@@ -1668,28 +1668,28 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>86</v>
+        <v>107.93</v>
       </c>
       <c r="E37" t="n">
-        <v>89.62</v>
+        <v>112.44</v>
       </c>
       <c r="F37" t="n">
-        <v>175.77</v>
+        <v>113.2</v>
       </c>
       <c r="G37" t="n">
-        <v>179.46</v>
+        <v>112.59</v>
       </c>
       <c r="H37" t="n">
-        <v>0.8559</v>
+        <v>0.9999</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0502</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0.0025</v>
+        <v>0.3351</v>
       </c>
     </row>
     <row r="38">
@@ -1702,28 +1702,28 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>111.84</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>112.64</v>
       </c>
       <c r="F38" t="n">
-        <v>224</v>
+        <v>112.53</v>
       </c>
       <c r="G38" t="n">
-        <v>224</v>
+        <v>114.2</v>
       </c>
       <c r="H38" t="n">
         <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>0.0327</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>0.4063</v>
       </c>
     </row>
     <row r="39">
@@ -1736,28 +1736,28 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>111.05</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>111.83</v>
       </c>
       <c r="F39" t="n">
-        <v>224</v>
+        <v>112.55</v>
       </c>
       <c r="G39" t="n">
-        <v>224</v>
+        <v>113.31</v>
       </c>
       <c r="H39" t="n">
-        <v>1</v>
+        <v>0.997</v>
       </c>
       <c r="I39" t="n">
-        <v>0.06510000000000001</v>
+        <v>0.0002</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>0.2628</v>
       </c>
     </row>
     <row r="40">
@@ -1770,28 +1770,28 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>108.77</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>112.43</v>
       </c>
       <c r="F40" t="n">
-        <v>224</v>
+        <v>112.33</v>
       </c>
       <c r="G40" t="n">
-        <v>224</v>
+        <v>112.86</v>
       </c>
       <c r="H40" t="n">
-        <v>0.0118</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="I40" t="n">
-        <v>0.2659</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0.0024</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1804,25 +1804,25 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>110.11</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>111.31</v>
       </c>
       <c r="F41" t="n">
-        <v>224</v>
+        <v>113.05</v>
       </c>
       <c r="G41" t="n">
-        <v>224</v>
+        <v>112.44</v>
       </c>
       <c r="H41" t="n">
-        <v>0.5724</v>
+        <v>0.7862</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0973</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -1841,25 +1841,25 @@
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>109.61</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>112.61</v>
       </c>
       <c r="F42" t="n">
-        <v>224</v>
+        <v>113.04</v>
       </c>
       <c r="G42" t="n">
-        <v>224</v>
+        <v>112.77</v>
       </c>
       <c r="H42" t="n">
-        <v>0.0157</v>
+        <v>0.9978</v>
       </c>
       <c r="I42" t="n">
-        <v>0.1197</v>
+        <v>0.0001</v>
       </c>
       <c r="J42" t="n">
-        <v>0.0015</v>
+        <v>0.2793</v>
       </c>
     </row>
     <row r="43">
@@ -1872,28 +1872,28 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>109.49</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>112.36</v>
       </c>
       <c r="F43" t="n">
-        <v>224</v>
+        <v>112.89</v>
       </c>
       <c r="G43" t="n">
-        <v>224</v>
+        <v>112.36</v>
       </c>
       <c r="H43" t="n">
-        <v>0.9906</v>
+        <v>0.9991</v>
       </c>
       <c r="I43" t="n">
-        <v>0.2101</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>0.5019</v>
       </c>
     </row>
     <row r="44">
@@ -1909,25 +1909,25 @@
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>109.1</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>112.64</v>
       </c>
       <c r="F44" t="n">
-        <v>224</v>
+        <v>114.25</v>
       </c>
       <c r="G44" t="n">
-        <v>224</v>
+        <v>113.4</v>
       </c>
       <c r="H44" t="n">
-        <v>0.6498</v>
+        <v>0.0001</v>
       </c>
       <c r="I44" t="n">
-        <v>0.1373</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>0.148</v>
       </c>
     </row>
     <row r="45">
@@ -1940,25 +1940,25 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>108.28</v>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>113.66</v>
       </c>
       <c r="F45" t="n">
-        <v>224</v>
+        <v>115.47</v>
       </c>
       <c r="G45" t="n">
-        <v>224</v>
+        <v>113.74</v>
       </c>
       <c r="H45" t="n">
-        <v>0.0238</v>
+        <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0.0891</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>

</xml_diff>